<commit_message>
29/july/2026 att. 2 Routines revised for unit conversion calculus. Added output file to .gitignore (should ignore the output spreadsheet this program generates. Check .gitignore whenever there are changes to main programs like main.py or routines.py)
</commit_message>
<xml_diff>
--- a/data/output/tabela_de_sais_concatenada.xlsx
+++ b/data/output/tabela_de_sais_concatenada.xlsx
@@ -729,7 +729,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>b_total (mol/kg)</t>
+          <t>b_total</t>
         </is>
       </c>
     </row>
@@ -8550,13 +8550,13 @@
         <v>0</v>
       </c>
       <c r="F264" t="n">
-        <v>0.09279636590074411</v>
+        <v>0.06704912422208589</v>
       </c>
       <c r="G264" t="n">
-        <v>0.9072036340992559</v>
+        <v>0.9329508757779141</v>
       </c>
       <c r="H264" t="n">
-        <v>5.677866420460327</v>
+        <v>3.989268947015426</v>
       </c>
     </row>
     <row r="265">
@@ -8577,16 +8577,16 @@
         <v>0.9869232667160128</v>
       </c>
       <c r="E265" t="n">
-        <v>0.699596479875854</v>
+        <v>0.08831233460161125</v>
       </c>
       <c r="F265" t="n">
-        <v>0.114901814379305</v>
+        <v>0.01450442900970296</v>
       </c>
       <c r="G265" t="n">
-        <v>0.185501705744841</v>
+        <v>0.8971832363886858</v>
       </c>
       <c r="H265" t="n">
-        <v>243.725660058305</v>
+        <v>6.361239727521758</v>
       </c>
     </row>
     <row r="266">
@@ -8607,16 +8607,16 @@
         <v>0.9869232667160128</v>
       </c>
       <c r="E266" t="n">
-        <v>0.7213024615163754</v>
+        <v>0.09005011374150375</v>
       </c>
       <c r="F266" t="n">
-        <v>0.08787544384968934</v>
+        <v>0.0109707011079845</v>
       </c>
       <c r="G266" t="n">
-        <v>0.1908220946339351</v>
+        <v>0.8989791851505118</v>
       </c>
       <c r="H266" t="n">
-        <v>235.3825918304396</v>
+        <v>6.237638683506662</v>
       </c>
     </row>
     <row r="267">
@@ -8637,16 +8637,16 @@
         <v>0.9869232667160128</v>
       </c>
       <c r="E267" t="n">
-        <v>0.8333308652855632</v>
+        <v>0.09302401414833508</v>
       </c>
       <c r="F267" t="n">
-        <v>0.06756386447707444</v>
+        <v>0.007542096599143512</v>
       </c>
       <c r="G267" t="n">
-        <v>0.09910527023736242</v>
+        <v>0.8994338892525214</v>
       </c>
       <c r="H267" t="n">
-        <v>504.5872584250056</v>
+        <v>6.206423278627589</v>
       </c>
     </row>
     <row r="268">
@@ -8667,16 +8667,16 @@
         <v>0.9869232667160128</v>
       </c>
       <c r="E268" t="n">
-        <v>0.8965405601933728</v>
+        <v>0.09522016250920992</v>
       </c>
       <c r="F268" t="n">
-        <v>0.03730291868192341</v>
+        <v>0.00396188431028092</v>
       </c>
       <c r="G268" t="n">
-        <v>0.06615652112470383</v>
+        <v>0.9008179531805092</v>
       </c>
       <c r="H268" t="n">
-        <v>783.5386326816827</v>
+        <v>6.111601334917133</v>
       </c>
     </row>
     <row r="269">
@@ -8696,10 +8696,18 @@
       <c r="D269" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E269" t="inlineStr"/>
-      <c r="F269" t="inlineStr"/>
-      <c r="G269" t="inlineStr"/>
-      <c r="H269" t="inlineStr"/>
+      <c r="E269" t="n">
+        <v>0.0981658717852128</v>
+      </c>
+      <c r="F269" t="n">
+        <v>0</v>
+      </c>
+      <c r="G269" t="n">
+        <v>0.9018341282147873</v>
+      </c>
+      <c r="H269" t="n">
+        <v>6.042168674698794</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -9584,13 +9592,13 @@
         <v>0</v>
       </c>
       <c r="F299" t="n">
-        <v>0.1016027485682283</v>
+        <v>0.07152867449024999</v>
       </c>
       <c r="G299" t="n">
-        <v>0.8983972514317717</v>
+        <v>0.9284713255097501</v>
       </c>
       <c r="H299" t="n">
-        <v>6.277634489654702</v>
+        <v>4.276324614352783</v>
       </c>
     </row>
     <row r="300">
@@ -9610,10 +9618,18 @@
       <c r="D300" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E300" t="inlineStr"/>
-      <c r="F300" t="inlineStr"/>
-      <c r="G300" t="inlineStr"/>
-      <c r="H300" t="inlineStr"/>
+      <c r="E300" t="n">
+        <v>0.09003706453597192</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0.01691928929438783</v>
+      </c>
+      <c r="G300" t="n">
+        <v>0.8930436461696402</v>
+      </c>
+      <c r="H300" t="n">
+        <v>6.648028734656937</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -9632,10 +9648,18 @@
       <c r="D301" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E301" t="inlineStr"/>
-      <c r="F301" t="inlineStr"/>
-      <c r="G301" t="inlineStr"/>
-      <c r="H301" t="inlineStr"/>
+      <c r="E301" t="n">
+        <v>0.09393009399992701</v>
+      </c>
+      <c r="F301" t="n">
+        <v>0.01194854356026697</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0.8941213624398061</v>
+      </c>
+      <c r="H301" t="n">
+        <v>6.573109338763505</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -9654,10 +9678,18 @@
       <c r="D302" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E302" t="inlineStr"/>
-      <c r="F302" t="inlineStr"/>
-      <c r="G302" t="inlineStr"/>
-      <c r="H302" t="inlineStr"/>
+      <c r="E302" t="n">
+        <v>0.09525527621317438</v>
+      </c>
+      <c r="F302" t="n">
+        <v>0.009111827746662157</v>
+      </c>
+      <c r="G302" t="n">
+        <v>0.8956328960401635</v>
+      </c>
+      <c r="H302" t="n">
+        <v>6.468336121144538</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -9676,10 +9708,18 @@
       <c r="D303" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E303" t="inlineStr"/>
-      <c r="F303" t="inlineStr"/>
-      <c r="G303" t="inlineStr"/>
-      <c r="H303" t="inlineStr"/>
+      <c r="E303" t="n">
+        <v>0.0978214071818788</v>
+      </c>
+      <c r="F303" t="n">
+        <v>0.00440409492708569</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0.8977744978910355</v>
+      </c>
+      <c r="H303" t="n">
+        <v>6.320493240567905</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -9698,10 +9738,18 @@
       <c r="D304" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E304" t="inlineStr"/>
-      <c r="F304" t="inlineStr"/>
-      <c r="G304" t="inlineStr"/>
-      <c r="H304" t="inlineStr"/>
+      <c r="E304" t="n">
+        <v>0.100547864762082</v>
+      </c>
+      <c r="F304" t="n">
+        <v>0.001692186390876834</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0.8977599488470411</v>
+      </c>
+      <c r="H304" t="n">
+        <v>6.321495236479115</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -9724,13 +9772,13 @@
         <v>0</v>
       </c>
       <c r="F305" t="n">
-        <v>0.1106188510346711</v>
+        <v>0.07588287253675204</v>
       </c>
       <c r="G305" t="n">
-        <v>0.8893811489653288</v>
+        <v>0.9241171274632479</v>
       </c>
       <c r="H305" t="n">
-        <v>6.903990843983419</v>
+        <v>4.558014755197853</v>
       </c>
     </row>
     <row r="306">
@@ -9750,10 +9798,18 @@
       <c r="D306" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E306" t="inlineStr"/>
-      <c r="F306" t="inlineStr"/>
-      <c r="G306" t="inlineStr"/>
-      <c r="H306" t="inlineStr"/>
+      <c r="E306" t="n">
+        <v>0.09267116669616399</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0.01691254673798606</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0.89041628656585</v>
+      </c>
+      <c r="H306" t="n">
+        <v>6.831434389469346</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -9772,10 +9828,18 @@
       <c r="D307" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E307" t="inlineStr"/>
-      <c r="F307" t="inlineStr"/>
-      <c r="G307" t="inlineStr"/>
-      <c r="H307" t="inlineStr"/>
+      <c r="E307" t="n">
+        <v>0.09489209417981619</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0.01197845381692465</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0.8931294520032592</v>
+      </c>
+      <c r="H307" t="n">
+        <v>6.642057162250612</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -9794,10 +9858,18 @@
       <c r="D308" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E308" t="inlineStr"/>
-      <c r="F308" t="inlineStr"/>
-      <c r="G308" t="inlineStr"/>
-      <c r="H308" t="inlineStr"/>
+      <c r="E308" t="n">
+        <v>0.09802257789909859</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0.009468268559736428</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0.8925091535411649</v>
+      </c>
+      <c r="H308" t="n">
+        <v>6.685252074697179</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -9816,10 +9888,18 @@
       <c r="D309" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E309" t="inlineStr"/>
-      <c r="F309" t="inlineStr"/>
-      <c r="G309" t="inlineStr"/>
-      <c r="H309" t="inlineStr"/>
+      <c r="E309" t="n">
+        <v>0.101408808356607</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0.004408085368591953</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0.894183106274801</v>
+      </c>
+      <c r="H309" t="n">
+        <v>6.568822573998205</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -9838,10 +9918,18 @@
       <c r="D310" t="n">
         <v>0.9869232667160128</v>
       </c>
-      <c r="E310" t="inlineStr"/>
-      <c r="F310" t="inlineStr"/>
-      <c r="G310" t="inlineStr"/>
-      <c r="H310" t="inlineStr"/>
+      <c r="E310" t="n">
+        <v>0.1042152723057443</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0.8957847276942557</v>
+      </c>
+      <c r="H310" t="n">
+        <v>6.457831325301205</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">

</xml_diff>